<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-05 Sarah laisse le temps à Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-05.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La pomme de Sarah</t>
+          <t>Sarah laisse le temps à Nina</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, goûter</t>
+          <t>cuisine, goûter, pomme, assiette ronde, nappe, frigo, évier, quartier, jus</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, Sarah, maman, papa</t>
+          <t>Sarah, Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Maman coupe la pomme. Sarah cherche ses mots. Raphaël attend. Pomme. Puis rouge. Ils croquent ensemble.</t>
+          <t>Ça sent la pomme près de l'évier. Sur le bord, un éclat d'assiette luit. Sarah veut aider Nina, maintenant. Elle dit le mot trop vite. Sourire parti. Papa s'accroupit. Elle ouvre la bouche, la referme, attend. Merci vécu. Deuxième ruse : le quartier glisse. Elle refuse de foncer. Un éclat d'assiette tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les pelures de pomme font une spirale. Elles sont vertes, un peu luisantes. La nappe a des petits carrés bleus. Le frigo fait un petit ronron. Un rayon pose un carré sur la table. Une mouche tapote la vitre, tout doux. C'est le goûter. J'ai coupé la pomme. Ça sent bon, hein ? Oui, papa. En ce moment, Raphaël est à table. Ses pieds touchent le barreau. Tu es bien assis, Raphaël ? Oui, papa. J'essuie le couteau. L'eau fait un petit bruit. Sarah est à côté. Elle veut parler. Elle cherche ses mots. Po... Raphaël connaît le mot. Il ouvre la bouche. On laisse le temps. On attend la fin de la phrase. Raphaël referme la bouche. Il pose ses mains. Il attend. Pomme. Puis un silence. Rouge. Rouge, oui. Bravo, Raphaël. Tu as laissé le temps. Tu as écouté jusqu'à la fin ? Oui, papa. Maman donne un quartier. Il est froid et lisse. Encore... Sarah cherche encore. Raphaël attend encore. Le frigo ronronne. Encore un morceau. Voici, Sarah. Tu as fini ta phrase. Ils croquent la pomme. Ça fait un petit bruit. C'est doux, la pomme ? Oui. Un peu sucré. Il y a... Sarah cherche encore un mot. Raphaël attend. Un pépin brille sur la nappe. Il y a un pépin. Un pépin, oui. Tu as laissé le temps, encore. Bravo. On met le pépin dans le bol ? Oui. Raphaël pousse le pépin. Le temps est doux. Raphaël écoute jusqu'à la fin. Tu veux un peu de jus ? Oui, maman. Le jus est jaune, un peu trouble. On boit sans se presser. C'est... Raphaël attend. C'est doux. Tu as encore laissé le temps.</t>
+          <t>Ça sent la pomme, près de l'évier. Ça sent bon, papa. Tu le sens, le fruit froid ? Oui, papa. L'eau tapote dans le fond. J'ai rincé la pomme. Elle brille, maman. Maman pose l'assiette ronde. L'assiette est froide, un peu lisse. Elle est froide. Tu la touches, Sarah ? Oui, du doigt. Sur le bord, un éclat d'assiette luit. Il brille, maman. Tu le vois, sur le bord ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur la nappe. La nappe gratte un peu. Elle gratte, papa. Tu t'assois, Sarah ? Un peu. Une miette dort sur la nappe. Une miette, maman. Elle est sèche ? Oui. Le frigo ronronne, tout près. Il ronronne, papa. Tu l'entends, le frigo ? Oui, il ronronne. Une goutte tombe dans l'évier. Ploc. C'est une goutte. Les pieds de Sarah touchent le barreau. Mes pieds, papa. Tu es bien assise, Sarah ? Oui, papa. Le bois du barreau est lisse. Il est lisse. Nina arrive près de la table. Ses chaussettes glissent sur le carreau. La pomme. Tu viens, Nina ? Oui. Maman pose des quartiers. Ils sont froids, un peu humides. Je veux aider, maintenant ! Tout de suite ? Oui, papa. En ce moment, Sarah tend un quartier. Tu le donnes à Nina ? Oui, maman. Nina prend le quartier. Elle ouvre la bouche. Po. Sarah connaît le mot. Elle ouvre la bouche. Pomme ! Nina baisse les yeux. Oh. Le sourire de Sarah disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Sarah ? Oui, papa. Tes mains sont froides, Sarah ? Un peu, maman. L'éclat d'assiette tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les pelures de pomme font une spirale. Elles sont vertes, un peu luisantes. La nappe a des petits carrés bleus. Le frigo fait un petit ronron. Un rayon pose un carré sur la table. Une mouche tapote la vitre, tout doux. C'est le goûter. J'ai coupé la pomme. Ça sent bon, hein ? Oui, papa. En ce moment, Raphaël est à table. Ses pieds touchent le barreau. Tu es bien assis, Raphaël ? Oui, papa. J'essuie le couteau. L'eau fait un petit bruit. Sarah est à côté. Elle veut parler. Elle cherche ses mots. Po... Raphaël connaît le mot. Il ouvre la bouche. On laisse le temps. On attend la fin de la phrase. Raphaël referme la bouche. Il pose ses mains. Il attend. Pomme. Puis un silence. Rouge. Rouge, oui. Bravo, Raphaël. Tu as laissé le temps. Tu as écouté jusqu'à la fin ? Oui, papa. Maman donne un quartier. Il est froid et lisse. Encore... Sarah cherche encore. Raphaël attend encore. Le frigo ronronne. Encore un morceau. Voici, Sarah. Tu as fini ta phrase. Ils croquent la pomme. Ça fait un petit bruit. C'est doux, la pomme ? Oui. Un peu sucré. Il y a... Sarah cherche encore un mot. Raphaël attend. Un pépin brille sur la nappe. Il y a un pépin. Un pépin, oui. Tu as laissé le temps, encore. Bravo. On met le pépin dans le bol ? Oui. Raphaël pousse le pépin. Le temps est doux. Raphaël écoute jusqu'à la fin. Tu veux un peu de jus ? Oui, maman. Le jus est jaune, un peu trouble. On boit sans se presser. C'est... Raphaël attend. C'est doux. Tu as encore laissé le temps.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ça sent la pomme, près de l'évier. Ça sent bon, papa. Tu le sens, le fruit froid ? Oui, papa. L'eau tapote dans le fond. J'ai rincé la pomme. Elle brille, maman. Maman pose l'assiette ronde. L'assiette est froide, un peu lisse. Elle est froide. Tu la touches, Sarah ? Oui, du doigt. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat d'assiette&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bord ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur la nappe. La nappe gratte un peu. Elle gratte, papa. Tu t'assois, Sarah ? Un peu. Une miette dort sur la nappe. Une miette, maman. Elle est sèche ? Oui. Le frigo ronronne, tout près. Il ronronne, papa. Tu l'entends, le frigo ? Oui, il ronronne. Une goutte tombe dans l'évier. Ploc. C'est une goutte. Les pieds de Sarah touchent le barreau. Mes pieds, papa. Tu es bien assise, Sarah ? Oui, papa. Le bois du barreau est lisse. Il est lisse. Nina arrive près de la table. Ses chaussettes glissent sur le carreau. La pomme. Tu viens, Nina ? Oui. Maman pose des quartiers. Ils sont froids, un peu humides. Je veux aider, maintenant ! Tout de suite ? Oui, papa. En ce moment, Sarah tend un quartier. Tu le donnes à Nina ? Oui, maman. Nina prend le quartier. Elle ouvre la bouche. Po. Sarah connaît le mot. Elle ouvre la bouche. Pomme ! Nina baisse les yeux. Oh. Le sourire de Sarah disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Sarah ? Oui, papa. Tes mains sont froides, Sarah ? Un peu, maman. L'éclat d'assiette tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Barbara est à table. C'est le goûter. Maman coupe la pomme. Nina veut parler. Nina cherche ses mots. Barbara attend. Elle laisse le temps. Nina dit : pomme. Puis elle dit : rouge. Barbara sourit. Barbara écoute jusqu'à la fin. Maman dit : tu as laissé le temps. Papa écoute aussi. Nina finit sa phrase. Barbara attend encore. Le temps est doux. Elles croquent la pomme.&lt;/slow&gt; [pause]</t>
+          <t>Ça sent la pomme, près de l'évier. Ça sent bon, papa. Tu le sens, le fruit froid ? Oui, papa. L'eau tapote dans le fond. J'ai rincé la pomme. Elle brille, maman. Maman pose l'assiette ronde. L'assiette est froide, un peu lisse. Elle est froide. Tu la touches, Sarah ? Oui, du doigt. Sur le bord, un &lt;emphasis&gt;éclat d'assiette&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bord ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur la nappe. La nappe gratte un peu. Elle gratte, papa. Tu t'assois, Sarah ? Un peu. Une miette dort sur la nappe. Une miette, maman. Elle est sèche ? Oui. Le frigo ronronne, tout près. Il ronronne, papa. Tu l'entends, le frigo ? Oui, il ronronne. Une goutte tombe dans l'évier. Ploc. C'est une goutte. Les pieds de Sarah touchent le barreau. Mes pieds, papa. Tu es bien assise, Sarah ? Oui, papa. Le bois du barreau est lisse. Il est lisse. Nina arrive près de la table. Ses chaussettes glissent sur le carreau. La pomme. Tu viens, Nina ? Oui. Maman pose des quartiers. Ils sont froids, un peu humides. Je veux aider, maintenant ! Tout de suite ? Oui, papa. En ce moment, Sarah tend un quartier. Tu le donnes à Nina ? Oui, maman. Nina prend le quartier. Elle ouvre la bouche. Po. Sarah connaît le mot. Elle ouvre la bouche. Pomme ! Nina baisse les yeux. Oh. Le sourire de Sarah disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Sarah ? Oui, papa. Tes mains sont froides, Sarah ? Un peu, maman. L'éclat d'assiette tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1273,28 +1273,32 @@
       <c r="AG2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'assiette</t>
+        </is>
+      </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1303,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1315,81 +1319,85 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_aider_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les pelures de pomme font une spirale.
-narrateur|Elles sont vertes, un peu luisantes.
-narrateur|La nappe a des petits carrés bleus.
-narrateur|Le frigo fait un petit ronron.
-narrateur|Un rayon pose un carré sur la table.
-narrateur|Une mouche tapote la vitre, tout doux.
-maman|C'est le goûter.
-maman|J'ai coupé la pomme.
-papa|Ça sent bon, hein ?
-enfant-m|Oui, papa.
-narrateur|En ce moment, Raphaël est à table.
-narrateur|Ses pieds touchent le barreau.
-papa|Tu es bien assis, Raphaël ?
-enfant-m|Oui, papa.
-maman|J'essuie le couteau.
-narrateur|L'eau fait un petit bruit.
-narrateur|Sarah est à côté.
-narrateur|Elle veut parler.
-narrateur|Elle cherche ses mots.
-copine|Po...
-narrateur|Raphaël connaît le mot.
-narrateur|Il ouvre la bouche.
-maman|On laisse le temps.
-maman|On attend la fin de la phrase.
-narrateur|Raphaël referme la bouche.
-narrateur|Il pose ses mains.
-narrateur|Il attend.
-copine|Pomme.
-narrateur|Puis un silence.
-copine|Rouge.
-enfant-m|Rouge, oui.
-maman|Bravo, Raphaël.
-maman|Tu as laissé le temps.
-papa|Tu as écouté jusqu'à la fin ?
-enfant-m|Oui, papa.
-narrateur|Maman donne un quartier.
-narrateur|Il est froid et lisse.
-copine|Encore...
-narrateur|Sarah cherche encore.
-narrateur|Raphaël attend encore.
-narrateur|Le frigo ronronne.
-copine|Encore un morceau.
-maman|Voici, Sarah.
-maman|Tu as fini ta phrase.
-narrateur|Ils croquent la pomme.
-narrateur|Ça fait un petit bruit.
-papa|C'est doux, la pomme ?
-enfant-m|Oui.
-enfant-m|Un peu sucré.
-copine|Il y a...
-narrateur|Sarah cherche encore un mot.
-narrateur|Raphaël attend.
-narrateur|Un pépin brille sur la nappe.
-copine|Il y a un pépin.
-enfant-m|Un pépin, oui.
-maman|Tu as laissé le temps, encore.
-maman|Bravo.
-papa|On met le pépin dans le bol ?
-enfant-m|Oui.
-narrateur|Raphaël pousse le pépin.
-narrateur|Le temps est doux.
-narrateur|Raphaël écoute jusqu'à la fin.
-maman|Tu veux un peu de jus ?
-enfant-m|Oui, maman.
-narrateur|Le jus est jaune, un peu trouble.
-papa|On boit sans se presser.
-copine|C'est...
-narrateur|Raphaël attend.
-copine|C'est doux.
-maman|Tu as encore laissé le temps.</t>
+          <t>narrateur|Ça sent la pomme, près de l'évier.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le fruit froid ?
+enfant-f|Oui, papa.
+narrateur|L'eau tapote dans le fond.
+maman|J'ai rincé la pomme.
+enfant-f|Elle brille, maman.
+narrateur|Maman pose l'assiette ronde.
+narrateur|L'assiette est froide, un peu lisse.
+enfant-f|Elle est froide.
+papa|Tu la touches, Sarah ?
+enfant-f|Oui, du doigt.
+narrateur|Sur le bord, un éclat d'assiette luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, sur le bord ?
+enfant-f|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse sur la nappe.
+narrateur|La nappe gratte un peu.
+enfant-f|Elle gratte, papa.
+maman|Tu t'assois, Sarah ?
+enfant-f|Un peu.
+narrateur|Une miette dort sur la nappe.
+enfant-f|Une miette, maman.
+maman|Elle est sèche ?
+enfant-f|Oui.
+narrateur|Le frigo ronronne, tout près.
+enfant-f|Il ronronne, papa.
+papa|Tu l'entends, le frigo ?
+enfant-f|Oui, il ronronne.
+narrateur|Une goutte tombe dans l'évier.
+enfant-f|Ploc.
+maman|C'est une goutte.
+narrateur|Les pieds de Sarah touchent le barreau.
+enfant-f|Mes pieds, papa.
+papa|Tu es bien assise, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le bois du barreau est lisse.
+enfant-f|Il est lisse.
+narrateur|Nina arrive près de la table.
+narrateur|Ses chaussettes glissent sur le carreau.
+copine|La pomme.
+enfant-f|Tu viens, Nina ?
+copine|Oui.
+narrateur|Maman pose des quartiers.
+narrateur|Ils sont froids, un peu humides.
+enfant-f|Je veux aider, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Sarah tend un quartier.
+maman|Tu le donnes à Nina ?
+enfant-f|Oui, maman.
+narrateur|Nina prend le quartier.
+narrateur|Elle ouvre la bouche.
+copine|Po.
+narrateur|Sarah connaît le mot.
+narrateur|Elle ouvre la bouche.
+enfant-f|Pomme !
+narrateur|Nina baisse les yeux.
+copine|Oh.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nina, Sarah ?
+enfant-f|Oui, papa.
+maman|Tes mains sont froides, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat d'assiette tremble, puis tient.</t>
         </is>
       </c>
     </row>
@@ -1416,17 +1424,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Sarah cherche ses mots. Que fait Raphaël ?</t>
+          <t>Nina cherche ses mots. Que fait Sarah ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah cherche ses mots. Que fait Raphaël ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina cherche ses &lt;emphasis level="moderate"&gt;mots&lt;/emphasis&gt;. Que fait Sarah ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nina cherche ses mots. Que fait Barbara ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina cherche ses &lt;emphasis&gt;mots&lt;/emphasis&gt;. Que fait Sarah ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1489,7 +1497,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1500,7 +1508,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1515,34 +1523,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>mots</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1557,7 +1569,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1567,13 +1579,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nina_cherche_ses_mots_que_fait_sarah; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Sarah cherche ses mots.
-narrateur|Que fait Raphaël ?</t>
+          <t>narrateur|Nina cherche ses mots.
+narrateur|Que fait Sarah ?</t>
         </is>
       </c>
     </row>
@@ -1600,17 +1612,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a laissé le temps. Sarah a fini sa phrase. On laisse le temps. Bravo, Raphaël. J'ai attendu.</t>
+          <t>Sarah veut aider, tout de suite. Je dis le mot, maintenant ! Elle avance trop vite vers Nina. Les mots se bousculent dans sa bouche. Attends. Nina recule d'un pas. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le quartier, un instant. Elle écoute le ronron du frigo. Tu veux aider Nina ? Papa reste à la même hauteur. Tu dis, Nina ? Nina ne dit rien, d'abord. Ses lèvres bougent, très lentement. Pomme. Pomme, oui. Merci, Sarah. Papa a vu les deux, près de l'assiette. Le quartier colle un peu, sous les doigts. Il est froid. Nina lèche une goutte. Sarah referme les lèvres. Rouge. Rouge, oui. Tu le vois, le quartier ? Oui, papa. Tu croques, Nina ? J'y vais. Ils croquent la pomme. Ça fait un petit bruit. Croc. Croc. C'est sucré, la pomme ? Nina ouvre la bouche. Su. Sarah referme les lèvres. Sucré. Sucré, oui. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. On reste près de l'assiette ? Oui. Tes mains sont au frais ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a laissé le temps. Sarah a fini sa phrase. On laisse le temps. Bravo, Raphaël. J'ai attendu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut aider, tout de suite. Je dis le mot, maintenant ! Elle avance trop vite vers Nina. Les mots se bousculent dans sa bouche. Attends. Nina recule d'un pas. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le &lt;emphasis level="moderate"&gt;quartier&lt;/emphasis&gt;, un instant. Elle écoute le ronron du frigo. Tu veux aider Nina ? Papa reste à la même hauteur. Tu dis, Nina ? Nina ne dit rien, d'abord. Ses lèvres bougent, très lentement. Pomme. Pomme, oui. Merci, Sarah. Papa a vu les deux, près de l'assiette. Le quartier colle un peu, sous les doigts. Il est froid. Nina lèche une goutte. Sarah referme les lèvres. Rouge. Rouge, oui. Tu le vois, le quartier ? Oui, papa. Tu croques, Nina ? J'y vais. Ils croquent la pomme. Ça fait un petit bruit. Croc. Croc. C'est sucré, la pomme ? Nina ouvre la bouche. Su. Sarah referme les lèvres. Sucré. Sucré, oui. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. On reste près de l'assiette ? Oui. Tes mains sont au frais ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Barbara a laissé le temps. Nina a fini sa phrase. Papa et maman ont vu.&lt;/slow&gt; [pause]</t>
+          <t>Sarah veut aider, tout de suite. Je dis le mot, maintenant ! Elle avance trop vite vers Nina. Les mots se bousculent dans sa bouche. Attends. Nina recule d'un pas. Oh. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le &lt;emphasis&gt;quartier&lt;/emphasis&gt;, un instant. Elle écoute le ronron du frigo. Tu veux aider Nina ? Papa reste à la même hauteur. Tu dis, Nina ? Nina ne dit rien, d'abord. Ses lèvres bougent, très lentement. Pomme. Pomme, oui. Merci, Sarah. Papa a vu les deux, près de l'assiette. Le quartier colle un peu, sous les doigts. Il est froid. Nina lèche une goutte. Sarah referme les lèvres. Rouge. Rouge, oui. Tu le vois, le quartier ? Oui, papa. Tu croques, Nina ? J'y vais. Ils croquent la pomme. Ça fait un petit bruit. Croc. Croc. C'est sucré, la pomme ? Nina ouvre la bouche. Su. Sarah referme les lèvres. Sucré. Sucré, oui. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. On reste près de l'assiette ? Oui. Tes mains sont au frais ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1657,18 +1669,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1689,28 +1701,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>quartier</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1719,10 +1735,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1731,20 +1747,63 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_referme_la_bouche_elle_attend; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a laissé le temps.
-narrateur|Sarah a fini sa phrase.
-maman|On laisse le temps.
-papa|Bravo, Raphaël.
-enfant-m|J'ai attendu.</t>
+          <t>narrateur|Sarah veut aider, tout de suite.
+enfant-f|Je dis le mot, maintenant !
+narrateur|Elle avance trop vite vers Nina.
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Attends.
+narrateur|Nina recule d'un pas.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le quartier, un instant.
+narrateur|Elle écoute le ronron du frigo.
+papa|Tu veux aider Nina ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Tu dis, Nina ?
+narrateur|Nina ne dit rien, d'abord.
+narrateur|Ses lèvres bougent, très lentement.
+copine|Pomme.
+enfant-f|Pomme, oui.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, près de l'assiette.
+maman|Le quartier colle un peu, sous les doigts.
+enfant-f|Il est froid.
+narrateur|Nina lèche une goutte.
+narrateur|Sarah referme les lèvres.
+copine|Rouge.
+enfant-f|Rouge, oui.
+papa|Tu le vois, le quartier ?
+enfant-f|Oui, papa.
+maman|Tu croques, Nina ?
+copine|J'y vais.
+narrateur|Ils croquent la pomme.
+narrateur|Ça fait un petit bruit.
+enfant-f|Croc.
+copine|Croc.
+papa|C'est sucré, la pomme ?
+narrateur|Nina ouvre la bouche.
+copine|Su.
+narrateur|Sarah referme les lèvres.
+copine|Sucré.
+enfant-f|Sucré, oui.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de l'assiette ?
+enfant-f|Oui.
+maman|Tes mains sont au frais ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1771,17 +1830,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël range les pelures. Tu mets ça dans le petit bol ? Oui, maman. Maman essuie la table. La nappe est propre, maintenant. On peut... Sarah cherche un mot. Raphaël attend. On peut boire. De l'eau, oui. Tu as encore attendu, Raphaël. Le carré de soleil a bougé.</t>
+          <t>Maman pose le verre de jus. Le verre est un peu flou. Le jus, maintenant ! Nina lève le verre. Le. Le quartier glisse sur l'assiette. Il glisse, maintenant ! Sarah avance les lèvres, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe l'assiette, un instant. Elle écoute le ronron du frigo. Sur le bord, un éclat d'assiette luit. Là, sur le bord. Tu dis, Nina ? Nina ne dit rien. Elle souffle, puis cherche. Il glisse. On pose le quartier ? Oui, papa. Sarah pousse le quartier. Nina le pose, sans se presser. Il tient. Il tient. Le jus est froid, Nina ? Un peu. Tu bois, Sarah ? Oui, maman. Ils boivent près de l'assiette. La nappe chatouille les poignets. C'est plus facile. Le frigo est calme ? Oui, papa. Un rayon passe sur le bord. Il allume l'assiette. Nina souffle sur le verre. Le jus. Le jus, oui. Le verre laisse un rond. Un rond d'eau.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël range les pelures. Tu mets ça dans le petit bol ? Oui, maman. Maman essuie la table. La nappe est propre, maintenant. On peut... Sarah cherche un mot. Raphaël attend. On peut boire. De l'eau, oui. Tu as encore attendu, Raphaël. Le carré de soleil a bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose le verre de jus. Le verre est un peu flou. Le jus, maintenant ! Nina lève le verre. Le. Le quartier glisse sur l'assiette. Il glisse, maintenant ! Sarah avance les lèvres, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe l'assiette, un instant. Elle écoute le ronron du frigo. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat d'assiette&lt;/emphasis&gt; luit. Là, sur le bord. Tu dis, Nina ? Nina ne dit rien. Elle souffle, puis cherche. Il glisse. On pose le quartier ? Oui, papa. Sarah pousse le quartier. Nina le pose, sans se presser. Il tient. Il tient. Le jus est froid, Nina ? Un peu. Tu bois, Sarah ? Oui, maman. Ils boivent près de l'assiette. La nappe chatouille les poignets. C'est plus facile. Le frigo est calme ? Oui, papa. Un rayon passe sur le bord. Il allume l'assiette. Nina souffle sur le verre. Le jus. Le jus, oui. Le verre laisse un rond. Un rond d'eau.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Barbara range les peaux. Maman essuie la table.&lt;/slow&gt; [pause]</t>
+          <t>Maman pose le verre de jus. Le verre est un peu flou. Le jus, maintenant ! Nina lève le verre. Le. Le quartier glisse sur l'assiette. Il glisse, maintenant ! Sarah avance les lèvres, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe l'assiette, un instant. Elle écoute le ronron du frigo. Sur le bord, un &lt;emphasis&gt;éclat d'assiette&lt;/emphasis&gt; luit. Là, sur le bord. Tu dis, Nina ? Nina ne dit rien. Elle souffle, puis cherche. Il glisse. On pose le quartier ? Oui, papa. Sarah pousse le quartier. Nina le pose, sans se presser. Il tient. Il tient. Le jus est froid, Nina ? Un peu. Tu bois, Sarah ? Oui, maman. Ils boivent près de l'assiette. La nappe chatouille les poignets. C'est plus facile. Le frigo est calme ? Oui, papa. Un rayon passe sur le bord. Il allume l'assiette. Nina souffle sur le verre. Le jus. Le jus, oui. Le verre laisse un rond. Un rond d'eau. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1828,18 +1887,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1860,28 +1919,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'assiette</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1890,10 +1953,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,23 +1965,57 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_quartier_glisse_elle_refuse_de_foncer; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël range les pelures.
-maman|Tu mets ça dans le petit bol ?
-enfant-m|Oui, maman.
-narrateur|Maman essuie la table.
-papa|La nappe est propre, maintenant.
-copine|On peut...
-narrateur|Sarah cherche un mot.
-narrateur|Raphaël attend.
-copine|On peut boire.
-papa|De l'eau, oui.
-papa|Tu as encore attendu, Raphaël.
-narrateur|Le carré de soleil a bougé.</t>
+          <t>narrateur|Maman pose le verre de jus.
+narrateur|Le verre est un peu flou.
+enfant-f|Le jus, maintenant !
+narrateur|Nina lève le verre.
+copine|Le.
+narrateur|Le quartier glisse sur l'assiette.
+enfant-f|Il glisse, maintenant !
+narrateur|Sarah avance les lèvres, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe l'assiette, un instant.
+narrateur|Elle écoute le ronron du frigo.
+narrateur|Sur le bord, un éclat d'assiette luit.
+enfant-f|Là, sur le bord.
+enfant-f|Tu dis, Nina ?
+narrateur|Nina ne dit rien.
+narrateur|Elle souffle, puis cherche.
+copine|Il glisse.
+papa|On pose le quartier ?
+enfant-f|Oui, papa.
+narrateur|Sarah pousse le quartier.
+narrateur|Nina le pose, sans se presser.
+enfant-f|Il tient.
+copine|Il tient.
+papa|Le jus est froid, Nina ?
+copine|Un peu.
+maman|Tu bois, Sarah ?
+enfant-f|Oui, maman.
+narrateur|Ils boivent près de l'assiette.
+narrateur|La nappe chatouille les poignets.
+enfant-f|C'est plus facile.
+papa|Le frigo est calme ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le bord.
+enfant-f|Il allume l'assiette.
+narrateur|Nina souffle sur le verre.
+copine|Le jus.
+enfant-f|Le jus, oui.
+narrateur|Le verre laisse un rond.
+enfant-f|Un rond d'eau.</t>
         </is>
       </c>
     </row>
@@ -1945,17 +2042,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. La spirale de pelures est dans le bol.</t>
+          <t>Ils restent près de l'assiette. Maman essuie un peu d'eau. La pomme a croqué, papa. Tu l'as vue, toi ? Oui, près de l'assiette. On est bien, ici. Sarah tapote le quartier du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le quartier est resté, Sarah. Oui, avec Nina. Le quartier est resté. Ça sent la pomme, un peu tiède. Et le jus, maman. Oui, dans l'air. La pomme reste dans l'assiette. Un éclat d'assiette tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. La spirale de pelures est dans le bol.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de l'assiette. Maman essuie un peu d'eau. La pomme a croqué, papa. Tu l'as vue, toi ? Oui, près de l'assiette. On est bien, ici. Sarah tapote le quartier du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le quartier est resté, Sarah. Oui, avec Nina. Le quartier est resté. Ça sent la pomme, un peu tiède. Et le jus, maman. Oui, dans l'air. La pomme reste dans l'assiette. Un &lt;emphasis level="moderate"&gt;éclat d'assiette&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de l'assiette. Maman essuie un peu d'eau. La pomme a croqué, papa. Tu l'as vue, toi ? Oui, près de l'assiette. On est bien, ici. Sarah tapote le quartier du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le quartier est resté, Sarah. Oui, avec Nina. Le quartier est resté. Ça sent la pomme, un peu tiède. Et le jus, maman. Oui, dans l'air. La pomme reste dans l'assiette. Un &lt;emphasis&gt;éclat d'assiette&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2002,7 +2099,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2010,7 +2107,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2022,12 +2119,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2036,14 +2133,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'assiette</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2055,11 +2156,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2068,26 +2169,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai attendu la fin.
-maman|Bravo.
-narrateur|La spirale de pelures est dans le bol.</t>
+          <t>narrateur|Ils restent près de l'assiette.
+narrateur|Maman essuie un peu d'eau.
+enfant-f|La pomme a croqué, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, près de l'assiette.
+maman|On est bien, ici.
+narrateur|Sarah tapote le quartier du doigt.
+enfant-f|Il a une trace d'eau.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le quartier est resté, Sarah.
+enfant-f|Oui, avec Nina.
+copine|Le quartier est resté.
+narrateur|Ça sent la pomme, un peu tiède.
+enfant-f|Et le jus, maman.
+maman|Oui, dans l'air.
+narrateur|La pomme reste dans l'assiette.
+narrateur|Un éclat d'assiette tient sur le bord.</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2172,6 +2292,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>